<commit_message>
29.07. dodati testovi placanja
</commit_message>
<xml_diff>
--- a/testdata/listForExecution.xlsx
+++ b/testdata/listForExecution.xlsx
@@ -4,14 +4,11 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="13128" windowHeight="8232"/>
+    <workbookView windowWidth="23040" windowHeight="8340"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$F$148</definedName>
-  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -30,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="906" uniqueCount="309">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="877" uniqueCount="304">
   <si>
     <t>TestName</t>
   </si>
@@ -878,85 +875,70 @@
     <t>C70900</t>
   </si>
   <si>
-    <t>Payments_Currency_Exchange_Pricelist_[WEB]-Overview</t>
+    <t>Payments_Domestic_Payments_Internal_Urgent_Payment_[WEB]</t>
   </si>
   <si>
     <t>C70901</t>
   </si>
   <si>
-    <t>Saving_Accounts_Transactions_Download_Option_[WEB]</t>
+    <t>Payments_Domestic_Payments_Internal_Non_Urgent_Payment_[WEB]</t>
   </si>
   <si>
     <t>C70902</t>
   </si>
   <si>
-    <t>Payments_Own_Account_Transfer_To_Loan_[WEB]</t>
+    <t>Payments_Domestic_Payments_External_Urgent_Payment_No_Model_[WEB]</t>
   </si>
   <si>
     <t>C70903</t>
   </si>
   <si>
-    <t>Payments_Own_Account_Transfer_From_Current_Foreign_Account_To_Current_Foreign_Account_[WEB]</t>
+    <t>Payments_Domestic_Payments_External_Urgent_Payment_Model11_Invalid_Bez_Poziva_Na_Broj_[WEB]</t>
   </si>
   <si>
     <t>C70904</t>
   </si>
   <si>
-    <t>Payments_Currency_Exchange_[WEB]-Buy_From_Payment</t>
+    <t>Payments_Domestic_Payments_External_Non_Urgent_Payment_Model11_[WEB]</t>
   </si>
   <si>
     <t>C70905</t>
   </si>
   <si>
-    <t>Payments_Currency_Exchange_[WEB]-Sell_From_Payment</t>
+    <t>Payments_Domestic_Payments_External_Urgent_Payment_Model97_Invalid_Bez_Poziva_Na_Broj_[WEB]</t>
   </si>
   <si>
     <t>C70906</t>
   </si>
   <si>
-    <t>Savings_Accounts_Transactions_Filter_By_Date_Date_Picker_[WEB]</t>
+    <t>Payments_Domestic_Payments_External_Non_Urgent_Payment_Model97_[WEB]</t>
   </si>
   <si>
     <t>C70907</t>
   </si>
   <si>
-    <t>Payments_Recipient_Template_List_[WEB]</t>
+    <t>Payments_Domestic_Payments_Budzetski_Urgent_Payment_Purpose_Code_289_Invalid_[WEB]</t>
   </si>
   <si>
     <t>C70908</t>
   </si>
   <si>
-    <t>Payments_Upcoming_Payments_Details_Of_Payments_Transaction_On_The_List_Of_Transaction_[WEB]</t>
+    <t>Payments_Domestic_Payments_Budzetski_Urgent_Payment_Without_Reference_Number_Invalid_[WEB]</t>
   </si>
   <si>
     <t>C70909</t>
   </si>
   <si>
+    <t>Payments_Domestic_Payments_Budzetski_Urgent_Payment_Model97_[WEB]</t>
+  </si>
+  <si>
     <t>C70910</t>
   </si>
   <si>
-    <t>Payments_Payments_Archive_Payments_Details_[WEB]</t>
+    <t>Payments_Domestic_Payments_Budzetski_Non_Urgent_Payment_Model97_[WEB]</t>
   </si>
   <si>
     <t>C70911</t>
-  </si>
-  <si>
-    <t>Current_Accounts_RSD_Statemants_List_[WEB]</t>
-  </si>
-  <si>
-    <t>C70912</t>
-  </si>
-  <si>
-    <t>Current_Foreign_Accounts_Statemants_List_[WEB]</t>
-  </si>
-  <si>
-    <t>C70913</t>
-  </si>
-  <si>
-    <t>Saving_Accounts_Accounts_Statemants_List_[WEB]</t>
-  </si>
-  <si>
-    <t>C70914</t>
   </si>
 </sst>
 </file>
@@ -1913,13 +1895,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:F151"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="5"/>
+  <dimension ref="A1:F148"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="91.1388888888889" customWidth="1"/>
+    <col min="1" max="1" width="94.1428571428571" customWidth="1"/>
+    <col min="2" max="2" width="11.7142857142857" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="1" spans="1:6">
+    <row r="1" spans="1:6">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1959,7 +1942,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" customFormat="1" spans="1:6">
+    <row r="3" spans="1:6">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -1979,7 +1962,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" customFormat="1" spans="1:6">
+    <row r="4" spans="1:6">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -1999,7 +1982,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" customFormat="1" spans="1:6">
+    <row r="5" spans="1:6">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -2019,7 +2002,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" customFormat="1" spans="1:6">
+    <row r="6" spans="1:6">
       <c r="A6" t="s">
         <v>18</v>
       </c>
@@ -2039,7 +2022,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" customFormat="1" spans="1:6">
+    <row r="7" spans="1:6">
       <c r="A7" t="s">
         <v>20</v>
       </c>
@@ -2059,7 +2042,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" customFormat="1" spans="1:6">
+    <row r="8" spans="1:6">
       <c r="A8" t="s">
         <v>22</v>
       </c>
@@ -2079,7 +2062,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" customFormat="1" spans="1:6">
+    <row r="9" spans="1:6">
       <c r="A9" t="s">
         <v>24</v>
       </c>
@@ -2099,7 +2082,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" customFormat="1" spans="1:6">
+    <row r="10" spans="1:6">
       <c r="A10" t="s">
         <v>26</v>
       </c>
@@ -2119,7 +2102,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" customFormat="1" spans="1:6">
+    <row r="11" spans="1:6">
       <c r="A11" t="s">
         <v>28</v>
       </c>
@@ -2139,7 +2122,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="12" customFormat="1" spans="1:6">
+    <row r="12" spans="1:6">
       <c r="A12" t="s">
         <v>30</v>
       </c>
@@ -2159,7 +2142,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" customFormat="1" spans="1:6">
+    <row r="13" spans="1:6">
       <c r="A13" t="s">
         <v>32</v>
       </c>
@@ -2179,7 +2162,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="14" customFormat="1" spans="1:6">
+    <row r="14" spans="1:6">
       <c r="A14" t="s">
         <v>34</v>
       </c>
@@ -2199,7 +2182,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="15" customFormat="1" spans="1:6">
+    <row r="15" spans="1:6">
       <c r="A15" t="s">
         <v>36</v>
       </c>
@@ -2219,7 +2202,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="16" customFormat="1" spans="1:6">
+    <row r="16" spans="1:6">
       <c r="A16" t="s">
         <v>38</v>
       </c>
@@ -2239,7 +2222,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="17" customFormat="1" spans="1:6">
+    <row r="17" spans="1:6">
       <c r="A17" t="s">
         <v>40</v>
       </c>
@@ -2259,7 +2242,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="18" customFormat="1" spans="1:6">
+    <row r="18" spans="1:6">
       <c r="A18" t="s">
         <v>42</v>
       </c>
@@ -2279,7 +2262,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="19" customFormat="1" spans="1:6">
+    <row r="19" spans="1:6">
       <c r="A19" t="s">
         <v>44</v>
       </c>
@@ -2299,7 +2282,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="20" customFormat="1" spans="1:6">
+    <row r="20" spans="1:6">
       <c r="A20" t="s">
         <v>46</v>
       </c>
@@ -2319,7 +2302,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="21" customFormat="1" spans="1:6">
+    <row r="21" spans="1:6">
       <c r="A21" t="s">
         <v>48</v>
       </c>
@@ -2339,7 +2322,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="22" customFormat="1" spans="1:6">
+    <row r="22" spans="1:6">
       <c r="A22" t="s">
         <v>50</v>
       </c>
@@ -2359,7 +2342,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="23" customFormat="1" spans="1:6">
+    <row r="23" spans="1:6">
       <c r="A23" t="s">
         <v>52</v>
       </c>
@@ -2379,7 +2362,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="24" customFormat="1" spans="1:6">
+    <row r="24" spans="1:6">
       <c r="A24" t="s">
         <v>54</v>
       </c>
@@ -2399,7 +2382,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="25" customFormat="1" spans="1:6">
+    <row r="25" spans="1:6">
       <c r="A25" t="s">
         <v>56</v>
       </c>
@@ -2419,7 +2402,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="26" customFormat="1" spans="1:6">
+    <row r="26" spans="1:6">
       <c r="A26" t="s">
         <v>58</v>
       </c>
@@ -2439,7 +2422,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="27" customFormat="1" spans="1:6">
+    <row r="27" spans="1:6">
       <c r="A27" t="s">
         <v>60</v>
       </c>
@@ -2459,7 +2442,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="28" customFormat="1" spans="1:6">
+    <row r="28" spans="1:6">
       <c r="A28" t="s">
         <v>62</v>
       </c>
@@ -2479,7 +2462,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="29" customFormat="1" spans="1:6">
+    <row r="29" spans="1:6">
       <c r="A29" t="s">
         <v>64</v>
       </c>
@@ -2499,7 +2482,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="30" customFormat="1" spans="1:6">
+    <row r="30" spans="1:6">
       <c r="A30" t="s">
         <v>66</v>
       </c>
@@ -2519,7 +2502,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="31" customFormat="1" spans="1:6">
+    <row r="31" spans="1:6">
       <c r="A31" t="s">
         <v>68</v>
       </c>
@@ -2539,7 +2522,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="32" customFormat="1" spans="1:6">
+    <row r="32" spans="1:6">
       <c r="A32" t="s">
         <v>70</v>
       </c>
@@ -2559,7 +2542,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="33" customFormat="1" spans="1:6">
+    <row r="33" spans="1:6">
       <c r="A33" t="s">
         <v>72</v>
       </c>
@@ -2579,7 +2562,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="34" customFormat="1" spans="1:6">
+    <row r="34" spans="1:6">
       <c r="A34" t="s">
         <v>74</v>
       </c>
@@ -2599,7 +2582,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="35" customFormat="1" spans="1:6">
+    <row r="35" spans="1:6">
       <c r="A35" t="s">
         <v>76</v>
       </c>
@@ -2619,7 +2602,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="36" customFormat="1" spans="1:6">
+    <row r="36" spans="1:6">
       <c r="A36" t="s">
         <v>78</v>
       </c>
@@ -2639,7 +2622,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="37" customFormat="1" spans="1:6">
+    <row r="37" spans="1:6">
       <c r="A37" t="s">
         <v>80</v>
       </c>
@@ -2659,7 +2642,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="38" customFormat="1" spans="1:6">
+    <row r="38" spans="1:6">
       <c r="A38" t="s">
         <v>82</v>
       </c>
@@ -2679,7 +2662,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="39" customFormat="1" spans="1:6">
+    <row r="39" spans="1:6">
       <c r="A39" t="s">
         <v>84</v>
       </c>
@@ -2699,7 +2682,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="40" customFormat="1" spans="1:6">
+    <row r="40" spans="1:6">
       <c r="A40" t="s">
         <v>86</v>
       </c>
@@ -2719,7 +2702,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="41" customFormat="1" spans="1:6">
+    <row r="41" spans="1:6">
       <c r="A41" t="s">
         <v>88</v>
       </c>
@@ -2739,7 +2722,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="42" customFormat="1" spans="1:6">
+    <row r="42" spans="1:6">
       <c r="A42" t="s">
         <v>90</v>
       </c>
@@ -2759,7 +2742,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="43" customFormat="1" spans="1:6">
+    <row r="43" spans="1:6">
       <c r="A43" t="s">
         <v>92</v>
       </c>
@@ -2779,7 +2762,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="44" customFormat="1" spans="1:6">
+    <row r="44" spans="1:6">
       <c r="A44" t="s">
         <v>94</v>
       </c>
@@ -2799,7 +2782,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="45" customFormat="1" spans="1:6">
+    <row r="45" spans="1:6">
       <c r="A45" t="s">
         <v>96</v>
       </c>
@@ -2819,7 +2802,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="46" customFormat="1" spans="1:6">
+    <row r="46" spans="1:6">
       <c r="A46" t="s">
         <v>98</v>
       </c>
@@ -2839,7 +2822,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="47" customFormat="1" spans="1:6">
+    <row r="47" spans="1:6">
       <c r="A47" t="s">
         <v>100</v>
       </c>
@@ -2859,7 +2842,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="48" customFormat="1" spans="1:6">
+    <row r="48" spans="1:6">
       <c r="A48" t="s">
         <v>102</v>
       </c>
@@ -2879,7 +2862,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="49" customFormat="1" spans="1:6">
+    <row r="49" spans="1:6">
       <c r="A49" t="s">
         <v>104</v>
       </c>
@@ -2899,7 +2882,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="50" customFormat="1" spans="1:6">
+    <row r="50" spans="1:6">
       <c r="A50" t="s">
         <v>106</v>
       </c>
@@ -2919,7 +2902,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="51" customFormat="1" spans="1:6">
+    <row r="51" spans="1:6">
       <c r="A51" t="s">
         <v>108</v>
       </c>
@@ -2939,7 +2922,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="52" customFormat="1" spans="1:6">
+    <row r="52" spans="1:6">
       <c r="A52" t="s">
         <v>110</v>
       </c>
@@ -2959,7 +2942,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="53" customFormat="1" spans="1:6">
+    <row r="53" spans="1:6">
       <c r="A53" t="s">
         <v>112</v>
       </c>
@@ -2979,7 +2962,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="54" customFormat="1" spans="1:6">
+    <row r="54" spans="1:6">
       <c r="A54" t="s">
         <v>114</v>
       </c>
@@ -2999,7 +2982,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="55" customFormat="1" spans="1:6">
+    <row r="55" spans="1:6">
       <c r="A55" t="s">
         <v>116</v>
       </c>
@@ -3019,7 +3002,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="56" customFormat="1" spans="1:6">
+    <row r="56" spans="1:6">
       <c r="A56" t="s">
         <v>118</v>
       </c>
@@ -3039,7 +3022,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="57" customFormat="1" spans="1:6">
+    <row r="57" spans="1:6">
       <c r="A57" t="s">
         <v>120</v>
       </c>
@@ -3059,7 +3042,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="58" customFormat="1" spans="1:6">
+    <row r="58" spans="1:6">
       <c r="A58" t="s">
         <v>122</v>
       </c>
@@ -3079,7 +3062,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="59" customFormat="1" spans="1:6">
+    <row r="59" spans="1:6">
       <c r="A59" t="s">
         <v>124</v>
       </c>
@@ -3099,7 +3082,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="60" customFormat="1" spans="1:6">
+    <row r="60" spans="1:6">
       <c r="A60" t="s">
         <v>126</v>
       </c>
@@ -3119,7 +3102,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="61" customFormat="1" spans="1:6">
+    <row r="61" spans="1:6">
       <c r="A61" t="s">
         <v>128</v>
       </c>
@@ -3139,7 +3122,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="62" customFormat="1" spans="1:6">
+    <row r="62" spans="1:6">
       <c r="A62" t="s">
         <v>130</v>
       </c>
@@ -3159,7 +3142,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="63" customFormat="1" spans="1:6">
+    <row r="63" spans="1:6">
       <c r="A63" t="s">
         <v>132</v>
       </c>
@@ -3179,7 +3162,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="64" customFormat="1" spans="1:6">
+    <row r="64" spans="1:6">
       <c r="A64" t="s">
         <v>134</v>
       </c>
@@ -3199,7 +3182,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="65" customFormat="1" spans="1:6">
+    <row r="65" spans="1:6">
       <c r="A65" t="s">
         <v>136</v>
       </c>
@@ -3219,7 +3202,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="66" customFormat="1" spans="1:6">
+    <row r="66" spans="1:6">
       <c r="A66" t="s">
         <v>138</v>
       </c>
@@ -3239,7 +3222,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="67" customFormat="1" spans="1:6">
+    <row r="67" spans="1:6">
       <c r="A67" t="s">
         <v>140</v>
       </c>
@@ -3259,7 +3242,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="68" customFormat="1" spans="1:6">
+    <row r="68" spans="1:6">
       <c r="A68" t="s">
         <v>142</v>
       </c>
@@ -3279,7 +3262,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="69" customFormat="1" spans="1:6">
+    <row r="69" spans="1:6">
       <c r="A69" t="s">
         <v>144</v>
       </c>
@@ -3299,7 +3282,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="70" customFormat="1" spans="1:6">
+    <row r="70" spans="1:6">
       <c r="A70" t="s">
         <v>146</v>
       </c>
@@ -3319,7 +3302,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="71" customFormat="1" spans="1:6">
+    <row r="71" spans="1:6">
       <c r="A71" t="s">
         <v>148</v>
       </c>
@@ -3339,7 +3322,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="72" customFormat="1" spans="1:6">
+    <row r="72" spans="1:6">
       <c r="A72" t="s">
         <v>150</v>
       </c>
@@ -3359,7 +3342,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="73" customFormat="1" spans="1:6">
+    <row r="73" spans="1:6">
       <c r="A73" t="s">
         <v>152</v>
       </c>
@@ -3379,7 +3362,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="74" customFormat="1" spans="1:6">
+    <row r="74" spans="1:6">
       <c r="A74" t="s">
         <v>154</v>
       </c>
@@ -3399,7 +3382,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="75" customFormat="1" spans="1:6">
+    <row r="75" spans="1:6">
       <c r="A75" t="s">
         <v>156</v>
       </c>
@@ -3419,7 +3402,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="76" customFormat="1" spans="1:6">
+    <row r="76" spans="1:6">
       <c r="A76" t="s">
         <v>158</v>
       </c>
@@ -3439,7 +3422,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="77" customFormat="1" spans="1:6">
+    <row r="77" spans="1:6">
       <c r="A77" t="s">
         <v>160</v>
       </c>
@@ -3459,7 +3442,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="78" customFormat="1" spans="1:6">
+    <row r="78" spans="1:6">
       <c r="A78" t="s">
         <v>162</v>
       </c>
@@ -3479,7 +3462,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="79" customFormat="1" spans="1:6">
+    <row r="79" spans="1:6">
       <c r="A79" t="s">
         <v>164</v>
       </c>
@@ -3499,7 +3482,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="80" customFormat="1" spans="1:6">
+    <row r="80" spans="1:6">
       <c r="A80" t="s">
         <v>166</v>
       </c>
@@ -3519,7 +3502,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="81" customFormat="1" spans="1:6">
+    <row r="81" spans="1:6">
       <c r="A81" t="s">
         <v>168</v>
       </c>
@@ -3539,7 +3522,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="82" customFormat="1" spans="1:6">
+    <row r="82" spans="1:6">
       <c r="A82" t="s">
         <v>170</v>
       </c>
@@ -3559,7 +3542,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="83" customFormat="1" spans="1:6">
+    <row r="83" spans="1:6">
       <c r="A83" t="s">
         <v>172</v>
       </c>
@@ -3579,7 +3562,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="84" customFormat="1" spans="1:6">
+    <row r="84" spans="1:6">
       <c r="A84" t="s">
         <v>174</v>
       </c>
@@ -3599,7 +3582,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="85" customFormat="1" spans="1:6">
+    <row r="85" spans="1:6">
       <c r="A85" t="s">
         <v>176</v>
       </c>
@@ -3619,7 +3602,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="86" customFormat="1" spans="1:6">
+    <row r="86" spans="1:6">
       <c r="A86" t="s">
         <v>178</v>
       </c>
@@ -3639,7 +3622,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="87" customFormat="1" spans="1:6">
+    <row r="87" spans="1:6">
       <c r="A87" t="s">
         <v>166</v>
       </c>
@@ -3659,7 +3642,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="88" customFormat="1" spans="1:6">
+    <row r="88" spans="1:6">
       <c r="A88" t="s">
         <v>181</v>
       </c>
@@ -3679,7 +3662,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="89" customFormat="1" spans="1:6">
+    <row r="89" spans="1:6">
       <c r="A89" t="s">
         <v>183</v>
       </c>
@@ -3699,7 +3682,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="90" customFormat="1" spans="1:6">
+    <row r="90" spans="1:6">
       <c r="A90" t="s">
         <v>185</v>
       </c>
@@ -3719,7 +3702,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="91" customFormat="1" spans="1:6">
+    <row r="91" spans="1:6">
       <c r="A91" t="s">
         <v>187</v>
       </c>
@@ -3739,7 +3722,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="92" customFormat="1" spans="1:6">
+    <row r="92" spans="1:6">
       <c r="A92" t="s">
         <v>189</v>
       </c>
@@ -3759,7 +3742,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="93" customFormat="1" spans="1:6">
+    <row r="93" spans="1:6">
       <c r="A93" t="s">
         <v>191</v>
       </c>
@@ -3779,7 +3762,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="94" customFormat="1" spans="1:6">
+    <row r="94" spans="1:6">
       <c r="A94" t="s">
         <v>193</v>
       </c>
@@ -3799,7 +3782,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="95" customFormat="1" spans="1:6">
+    <row r="95" spans="1:6">
       <c r="A95" t="s">
         <v>195</v>
       </c>
@@ -3819,7 +3802,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="96" customFormat="1" spans="1:6">
+    <row r="96" spans="1:6">
       <c r="A96" t="s">
         <v>197</v>
       </c>
@@ -3839,7 +3822,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="97" customFormat="1" spans="1:6">
+    <row r="97" spans="1:6">
       <c r="A97" t="s">
         <v>199</v>
       </c>
@@ -3859,7 +3842,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="98" customFormat="1" spans="1:6">
+    <row r="98" spans="1:6">
       <c r="A98" t="s">
         <v>201</v>
       </c>
@@ -3879,7 +3862,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="99" customFormat="1" spans="1:6">
+    <row r="99" spans="1:6">
       <c r="A99" t="s">
         <v>203</v>
       </c>
@@ -3899,7 +3882,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="100" customFormat="1" spans="1:6">
+    <row r="100" spans="1:6">
       <c r="A100" t="s">
         <v>205</v>
       </c>
@@ -3919,7 +3902,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="101" customFormat="1" spans="1:6">
+    <row r="101" spans="1:6">
       <c r="A101" t="s">
         <v>207</v>
       </c>
@@ -3939,7 +3922,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="102" customFormat="1" spans="1:6">
+    <row r="102" spans="1:6">
       <c r="A102" t="s">
         <v>209</v>
       </c>
@@ -3959,7 +3942,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="103" customFormat="1" spans="1:6">
+    <row r="103" spans="1:6">
       <c r="A103" t="s">
         <v>211</v>
       </c>
@@ -3979,7 +3962,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="104" customFormat="1" spans="1:6">
+    <row r="104" spans="1:6">
       <c r="A104" t="s">
         <v>213</v>
       </c>
@@ -3999,7 +3982,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="105" customFormat="1" spans="1:6">
+    <row r="105" spans="1:6">
       <c r="A105" t="s">
         <v>215</v>
       </c>
@@ -4019,7 +4002,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="106" customFormat="1" spans="1:6">
+    <row r="106" spans="1:6">
       <c r="A106" t="s">
         <v>217</v>
       </c>
@@ -4039,7 +4022,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="107" customFormat="1" spans="1:6">
+    <row r="107" spans="1:6">
       <c r="A107" t="s">
         <v>219</v>
       </c>
@@ -4059,7 +4042,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="108" customFormat="1" spans="1:6">
+    <row r="108" spans="1:6">
       <c r="A108" t="s">
         <v>221</v>
       </c>
@@ -4079,7 +4062,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="109" customFormat="1" spans="1:6">
+    <row r="109" spans="1:6">
       <c r="A109" t="s">
         <v>223</v>
       </c>
@@ -4099,7 +4082,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="110" customFormat="1" spans="1:6">
+    <row r="110" spans="1:6">
       <c r="A110" t="s">
         <v>225</v>
       </c>
@@ -4119,7 +4102,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="111" customFormat="1" spans="1:6">
+    <row r="111" spans="1:6">
       <c r="A111" t="s">
         <v>227</v>
       </c>
@@ -4139,7 +4122,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="112" customFormat="1" spans="1:6">
+    <row r="112" spans="1:6">
       <c r="A112" t="s">
         <v>229</v>
       </c>
@@ -4159,7 +4142,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="113" customFormat="1" spans="1:6">
+    <row r="113" spans="1:6">
       <c r="A113" t="s">
         <v>231</v>
       </c>
@@ -4179,7 +4162,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="114" customFormat="1" spans="1:6">
+    <row r="114" spans="1:6">
       <c r="A114" t="s">
         <v>233</v>
       </c>
@@ -4199,7 +4182,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="115" customFormat="1" spans="1:6">
+    <row r="115" spans="1:6">
       <c r="A115" t="s">
         <v>235</v>
       </c>
@@ -4219,7 +4202,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="116" customFormat="1" spans="1:6">
+    <row r="116" spans="1:6">
       <c r="A116" t="s">
         <v>237</v>
       </c>
@@ -4239,7 +4222,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="117" customFormat="1" spans="1:6">
+    <row r="117" spans="1:6">
       <c r="A117" t="s">
         <v>239</v>
       </c>
@@ -4259,7 +4242,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="118" customFormat="1" spans="1:6">
+    <row r="118" spans="1:6">
       <c r="A118" t="s">
         <v>241</v>
       </c>
@@ -4279,7 +4262,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="119" customFormat="1" spans="1:6">
+    <row r="119" spans="1:6">
       <c r="A119" t="s">
         <v>243</v>
       </c>
@@ -4299,7 +4282,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="120" customFormat="1" spans="1:6">
+    <row r="120" spans="1:6">
       <c r="A120" t="s">
         <v>245</v>
       </c>
@@ -4319,7 +4302,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="121" customFormat="1" spans="1:6">
+    <row r="121" spans="1:6">
       <c r="A121" t="s">
         <v>247</v>
       </c>
@@ -4339,7 +4322,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="122" customFormat="1" spans="1:6">
+    <row r="122" spans="1:6">
       <c r="A122" t="s">
         <v>249</v>
       </c>
@@ -4359,7 +4342,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="123" customFormat="1" spans="1:6">
+    <row r="123" spans="1:6">
       <c r="A123" t="s">
         <v>251</v>
       </c>
@@ -4379,7 +4362,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="124" customFormat="1" spans="1:6">
+    <row r="124" spans="1:6">
       <c r="A124" t="s">
         <v>253</v>
       </c>
@@ -4399,7 +4382,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="125" customFormat="1" spans="1:6">
+    <row r="125" spans="1:6">
       <c r="A125" t="s">
         <v>255</v>
       </c>
@@ -4419,7 +4402,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="126" customFormat="1" spans="1:6">
+    <row r="126" spans="1:6">
       <c r="A126" t="s">
         <v>257</v>
       </c>
@@ -4439,7 +4422,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="127" customFormat="1" spans="1:6">
+    <row r="127" spans="1:6">
       <c r="A127" t="s">
         <v>259</v>
       </c>
@@ -4459,7 +4442,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="128" customFormat="1" spans="1:6">
+    <row r="128" spans="1:6">
       <c r="A128" t="s">
         <v>261</v>
       </c>
@@ -4479,7 +4462,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="129" customFormat="1" spans="1:6">
+    <row r="129" spans="1:6">
       <c r="A129" t="s">
         <v>263</v>
       </c>
@@ -4499,7 +4482,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="130" customFormat="1" spans="1:6">
+    <row r="130" spans="1:6">
       <c r="A130" t="s">
         <v>265</v>
       </c>
@@ -4519,7 +4502,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="131" customFormat="1" spans="1:6">
+    <row r="131" spans="1:6">
       <c r="A131" t="s">
         <v>267</v>
       </c>
@@ -4539,7 +4522,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="132" customFormat="1" spans="1:6">
+    <row r="132" spans="1:6">
       <c r="A132" t="s">
         <v>269</v>
       </c>
@@ -4559,7 +4542,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="133" customFormat="1" spans="1:6">
+    <row r="133" spans="1:6">
       <c r="A133" t="s">
         <v>271</v>
       </c>
@@ -4659,15 +4642,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="138" customFormat="1" spans="1:6">
+    <row r="138" spans="1:6">
       <c r="A138" t="s">
         <v>282</v>
       </c>
       <c r="B138" s="2" t="s">
         <v>283</v>
       </c>
-      <c r="C138" s="1" t="s">
-        <v>8</v>
+      <c r="C138" s="1">
+        <v>3</v>
       </c>
       <c r="D138" s="1" t="s">
         <v>9</v>
@@ -4679,15 +4662,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="139" customFormat="1" spans="1:6">
+    <row r="139" spans="1:6">
       <c r="A139" t="s">
         <v>284</v>
       </c>
       <c r="B139" s="2" t="s">
         <v>285</v>
       </c>
-      <c r="C139" s="1" t="s">
-        <v>8</v>
+      <c r="C139" s="1">
+        <v>3</v>
       </c>
       <c r="D139" s="1" t="s">
         <v>9</v>
@@ -4699,15 +4682,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="140" customFormat="1" spans="1:6">
+    <row r="140" spans="1:6">
       <c r="A140" t="s">
         <v>286</v>
       </c>
       <c r="B140" s="2" t="s">
         <v>287</v>
       </c>
-      <c r="C140" s="1" t="s">
-        <v>8</v>
+      <c r="C140" s="1">
+        <v>3</v>
       </c>
       <c r="D140" s="1" t="s">
         <v>9</v>
@@ -4719,15 +4702,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="141" customFormat="1" spans="1:6">
+    <row r="141" spans="1:6">
       <c r="A141" t="s">
         <v>288</v>
       </c>
       <c r="B141" s="2" t="s">
         <v>289</v>
       </c>
-      <c r="C141" s="1" t="s">
-        <v>8</v>
+      <c r="C141" s="1">
+        <v>3</v>
       </c>
       <c r="D141" s="1" t="s">
         <v>9</v>
@@ -4739,15 +4722,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="142" customFormat="1" spans="1:6">
+    <row r="142" spans="1:6">
       <c r="A142" t="s">
         <v>290</v>
       </c>
       <c r="B142" s="2" t="s">
         <v>291</v>
       </c>
-      <c r="C142" s="1" t="s">
-        <v>8</v>
+      <c r="C142" s="1">
+        <v>3</v>
       </c>
       <c r="D142" s="1" t="s">
         <v>9</v>
@@ -4759,15 +4742,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="143" customFormat="1" spans="1:6">
+    <row r="143" spans="1:6">
       <c r="A143" t="s">
         <v>292</v>
       </c>
       <c r="B143" s="2" t="s">
         <v>293</v>
       </c>
-      <c r="C143" s="1" t="s">
-        <v>8</v>
+      <c r="C143" s="1">
+        <v>3</v>
       </c>
       <c r="D143" s="1" t="s">
         <v>9</v>
@@ -4779,15 +4762,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="144" customFormat="1" spans="1:6">
+    <row r="144" spans="1:6">
       <c r="A144" t="s">
         <v>294</v>
       </c>
       <c r="B144" s="2" t="s">
         <v>295</v>
       </c>
-      <c r="C144" s="1" t="s">
-        <v>8</v>
+      <c r="C144" s="1">
+        <v>3</v>
       </c>
       <c r="D144" s="1" t="s">
         <v>9</v>
@@ -4799,15 +4782,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="145" customFormat="1" spans="1:6">
+    <row r="145" spans="1:6">
       <c r="A145" t="s">
         <v>296</v>
       </c>
       <c r="B145" s="2" t="s">
         <v>297</v>
       </c>
-      <c r="C145" s="1" t="s">
-        <v>8</v>
+      <c r="C145" s="1">
+        <v>3</v>
       </c>
       <c r="D145" s="1" t="s">
         <v>9</v>
@@ -4819,15 +4802,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="146" customFormat="1" spans="1:6">
+    <row r="146" spans="1:6">
       <c r="A146" t="s">
         <v>298</v>
       </c>
       <c r="B146" s="2" t="s">
         <v>299</v>
       </c>
-      <c r="C146" s="1" t="s">
-        <v>8</v>
+      <c r="C146" s="1">
+        <v>3</v>
       </c>
       <c r="D146" s="1" t="s">
         <v>9</v>
@@ -4839,15 +4822,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="147" customFormat="1" spans="1:6">
+    <row r="147" spans="1:6">
       <c r="A147" t="s">
-        <v>280</v>
+        <v>300</v>
       </c>
       <c r="B147" s="2" t="s">
-        <v>300</v>
-      </c>
-      <c r="C147" s="1" t="s">
-        <v>8</v>
+        <v>301</v>
+      </c>
+      <c r="C147" s="1">
+        <v>3</v>
       </c>
       <c r="D147" s="1" t="s">
         <v>9</v>
@@ -4859,15 +4842,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="148" customFormat="1" spans="1:6">
+    <row r="148" spans="1:6">
       <c r="A148" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B148" s="2" t="s">
-        <v>302</v>
-      </c>
-      <c r="C148" s="1" t="s">
-        <v>8</v>
+        <v>303</v>
+      </c>
+      <c r="C148" s="1">
+        <v>3</v>
       </c>
       <c r="D148" s="1" t="s">
         <v>9</v>
@@ -4879,103 +4862,9 @@
         <v>11</v>
       </c>
     </row>
-    <row r="149" customFormat="1" spans="1:6">
-      <c r="A149" t="s">
-        <v>303</v>
-      </c>
-      <c r="B149" s="2" t="s">
-        <v>304</v>
-      </c>
-      <c r="C149" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D149" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E149" t="s">
-        <v>10</v>
-      </c>
-      <c r="F149" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="150" customFormat="1" spans="1:6">
-      <c r="A150" t="s">
-        <v>305</v>
-      </c>
-      <c r="B150" s="2" t="s">
-        <v>306</v>
-      </c>
-      <c r="C150" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D150" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E150" t="s">
-        <v>10</v>
-      </c>
-      <c r="F150" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="151" customFormat="1" spans="1:6">
-      <c r="A151" t="s">
-        <v>307</v>
-      </c>
-      <c r="B151" s="2" t="s">
-        <v>308</v>
-      </c>
-      <c r="C151" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D151" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E151" t="s">
-        <v>10</v>
-      </c>
-      <c r="F151" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:F148" etc:filterBottomFollowUsedRange="0">
-    <extLst/>
-  </autoFilter>
-  <conditionalFormatting sqref="A35">
-    <cfRule type="duplicateValues" dxfId="0" priority="16"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A69">
-    <cfRule type="duplicateValues" dxfId="0" priority="12"/>
-    <cfRule type="duplicateValues" dxfId="0" priority="11"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A74">
-    <cfRule type="duplicateValues" dxfId="0" priority="8"/>
-    <cfRule type="duplicateValues" dxfId="0" priority="7"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A75">
-    <cfRule type="duplicateValues" dxfId="0" priority="6"/>
-    <cfRule type="duplicateValues" dxfId="0" priority="5"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A80">
-    <cfRule type="duplicateValues" dxfId="0" priority="2"/>
+  <conditionalFormatting sqref="B$1:B$1048576">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A70:A71">
-    <cfRule type="duplicateValues" dxfId="0" priority="10"/>
-    <cfRule type="duplicateValues" dxfId="0" priority="9"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A78:A79">
-    <cfRule type="duplicateValues" dxfId="0" priority="4"/>
-    <cfRule type="duplicateValues" dxfId="0" priority="3"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B$1:B$1048576">
-    <cfRule type="duplicateValues" dxfId="0" priority="14"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A1:A68 A81:A1048576 A76:A77 A72:A73">
-    <cfRule type="duplicateValues" dxfId="0" priority="15"/>
-    <cfRule type="duplicateValues" dxfId="0" priority="13"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>

</xml_diff>

<commit_message>
29.07. dodata 3 testa external placanja
</commit_message>
<xml_diff>
--- a/testdata/listForExecution.xlsx
+++ b/testdata/listForExecution.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="877" uniqueCount="304">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="892" uniqueCount="310">
   <si>
     <t>TestName</t>
   </si>
@@ -939,6 +939,24 @@
   </si>
   <si>
     <t>C70911</t>
+  </si>
+  <si>
+    <t>Payments_Domestic_Payments_External_Urgent_Payment_Model97_[WEB]</t>
+  </si>
+  <si>
+    <t>C70912</t>
+  </si>
+  <si>
+    <t>Payments_Domestic_Payments_External_Urgent_Payment_Model11_[WEB]</t>
+  </si>
+  <si>
+    <t>C70913</t>
+  </si>
+  <si>
+    <t>Payments_Domestic_Payments_External_Non_Urgent_Payment_No_Model_[WEB]</t>
+  </si>
+  <si>
+    <t>C70914</t>
   </si>
 </sst>
 </file>
@@ -1895,7 +1913,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:F148"/>
+  <dimension ref="A1:F151"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" width="94.1428571428571" customWidth="1"/>
@@ -4862,6 +4880,66 @@
         <v>11</v>
       </c>
     </row>
+    <row r="149" spans="1:6">
+      <c r="A149" t="s">
+        <v>304</v>
+      </c>
+      <c r="B149" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="C149" s="1">
+        <v>3</v>
+      </c>
+      <c r="D149" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E149" t="s">
+        <v>10</v>
+      </c>
+      <c r="F149" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="150" spans="1:6">
+      <c r="A150" t="s">
+        <v>306</v>
+      </c>
+      <c r="B150" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="C150" s="1">
+        <v>3</v>
+      </c>
+      <c r="D150" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E150" t="s">
+        <v>10</v>
+      </c>
+      <c r="F150" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="151" spans="1:6">
+      <c r="A151" t="s">
+        <v>308</v>
+      </c>
+      <c r="B151" s="2" t="s">
+        <v>309</v>
+      </c>
+      <c r="C151" s="1">
+        <v>3</v>
+      </c>
+      <c r="D151" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E151" t="s">
+        <v>10</v>
+      </c>
+      <c r="F151" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="B$1:B$1048576">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>

</xml_diff>